<commit_message>
Colonne email dans le circuit Excel et l'import de comptes web
L'e-mail (identifiant de connexion Odoo) devient la clé de jointure : colonne
email dans column_plan (modèle + import), report depuis l'export Odoo dans
import_odoo.py, et l'import de comptes de la webapp accepte directement la
feuille Candidats (en-tête nom_prenom, libellé de département converti en id
du profil). Modèles d'exemple régénérés.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/enset/dossiers-u4.xlsx
+++ b/examples/enset/dossiers-u4.xlsx
@@ -617,29 +617,30 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T5"/>
+  <dimension ref="A1:U5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="32" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
     <col width="32" customWidth="1" min="8" max="8"/>
     <col width="32" customWidth="1" min="9" max="9"/>
     <col width="32" customWidth="1" min="10" max="10"/>
-    <col width="29" customWidth="1" min="11" max="11"/>
-    <col width="22" customWidth="1" min="12" max="12"/>
-    <col width="30" customWidth="1" min="13" max="13"/>
-    <col width="32" customWidth="1" min="14" max="14"/>
+    <col width="32" customWidth="1" min="11" max="11"/>
+    <col width="29" customWidth="1" min="12" max="12"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="30" customWidth="1" min="14" max="14"/>
     <col width="32" customWidth="1" min="15" max="15"/>
     <col width="32" customWidth="1" min="16" max="16"/>
-    <col width="27" customWidth="1" min="17" max="17"/>
-    <col width="24" customWidth="1" min="18" max="18"/>
-    <col width="20" customWidth="1" min="19" max="19"/>
-    <col width="19" customWidth="1" min="20" max="20"/>
+    <col width="32" customWidth="1" min="17" max="17"/>
+    <col width="27" customWidth="1" min="18" max="18"/>
+    <col width="24" customWidth="1" min="19" max="19"/>
+    <col width="20" customWidth="1" min="20" max="20"/>
+    <col width="19" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -650,95 +651,100 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>email</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>nom_prenom</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>population</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>departement</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>pays_destination</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>duree_jours</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>inscription_doctorat.inscription (qte)</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>penalite_beneficies_3ans (n manuel)</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>projet_startup_incubateur (Oui/Non)</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>structures_accompagnement.attestation (qte)</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>prix_distinctions (Oui/Non)</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>livre_isbn (Oui/Non)</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>livre_isbn (bonus 1 Oui/Non)</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>polycopie_pedagogique (Oui/Non)</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>polycopie_pedagogique (bonus 1 Oui/Non)</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>polycopie_pedagogique (bonus 2 Oui/Non)</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>poste_superieur (Oui/Non)</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>montant_indemnite (DA)</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>billet_estime (DA)</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>frais_divers (DA)</t>
         </is>
@@ -750,41 +756,41 @@
           <t>D101</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Bouzid Sara</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>doctorant_non_salarie</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Département de Technologie</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>France</t>
         </is>
       </c>
-      <c r="F2" t="n">
+      <c r="G2" t="n">
         <v>21</v>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>3</v>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Oui</t>
         </is>
       </c>
-      <c r="S2" t="n">
+      <c r="T2" t="n">
         <v>95000</v>
       </c>
-      <c r="T2" t="n">
+      <c r="U2" t="n">
         <v>28000</v>
       </c>
     </row>
@@ -794,44 +800,44 @@
           <t>D102</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Khelifi Mohamed</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="D3" t="inlineStr">
         <is>
           <t>doctorant_non_salarie</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Département de Technologie</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>Tunisie</t>
         </is>
       </c>
-      <c r="F3" t="n">
+      <c r="G3" t="n">
         <v>30</v>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" t="n">
         <v>4</v>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
-      <c r="J3" t="n">
+      <c r="K3" t="n">
         <v>1</v>
       </c>
-      <c r="S3" t="n">
+      <c r="T3" t="n">
         <v>38000</v>
       </c>
-      <c r="T3" t="n">
+      <c r="U3" t="n">
         <v>12000</v>
       </c>
     </row>
@@ -841,41 +847,41 @@
           <t>D103</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Aissaoui Rym</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>doctorant_non_salarie</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>Département de Mathématiques et Informatique</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>Espagne</t>
         </is>
       </c>
-      <c r="F4" t="n">
+      <c r="G4" t="n">
         <v>15</v>
       </c>
-      <c r="G4" t="n">
+      <c r="H4" t="n">
         <v>2</v>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
-      <c r="S4" t="n">
+      <c r="T4" t="n">
         <v>88000</v>
       </c>
-      <c r="T4" t="n">
+      <c r="U4" t="n">
         <v>26000</v>
       </c>
     </row>
@@ -885,63 +891,60 @@
           <t>E201</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Ziani Hocine</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>maitre_assistant</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>Département de Physique et Chimie</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>Japon</t>
         </is>
       </c>
-      <c r="F5" t="n">
+      <c r="G5" t="n">
         <v>15</v>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>Non</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
+      <c r="O5" t="inlineStr">
         <is>
           <t>Oui</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr">
+      <c r="P5" t="inlineStr">
         <is>
           <t>Oui</t>
         </is>
       </c>
-      <c r="S5" t="n">
+      <c r="T5" t="n">
         <v>460000</v>
       </c>
-      <c r="T5" t="n">
+      <c r="U5" t="n">
         <v>35000</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="10">
-    <dataValidation sqref="C2:C500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="D2:D500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>=Listes!$A$2:$A$4</formula1>
     </dataValidation>
-    <dataValidation sqref="D2:D500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="E2:E500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>=Listes!$B$2:$B$5</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>=Listes!$C$2:$C$3</formula1>
-    </dataValidation>
-    <dataValidation sqref="K2:K500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>=Listes!$C$2:$C$3</formula1>
     </dataValidation>
     <dataValidation sqref="L2:L500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
@@ -960,6 +963,9 @@
       <formula1>=Listes!$C$2:$C$3</formula1>
     </dataValidation>
     <dataValidation sqref="Q2:Q500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+      <formula1>=Listes!$C$2:$C$3</formula1>
+    </dataValidation>
+    <dataValidation sqref="R2:R500" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>=Listes!$C$2:$C$3</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>